<commit_message>
feat(deploy): update G7 official match reports & votes, FotMob xG+xA stats, 48 official injuries, tactical neutralizations & G8 4-source consensus lineups
</commit_message>
<xml_diff>
--- a/data/metriche_predittive_algoritmo.xlsx
+++ b/data/metriche_predittive_algoritmo.xlsx
@@ -433,7 +433,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="14">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -463,12 +463,6 @@
       <name val="Segoe UI"/>
       <family val="0"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
@@ -644,95 +638,95 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1533,11 +1527,11 @@
   <dimension ref="A1:E8"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="55"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="45"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="18"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>